<commit_message>
Fix distributor conflation and generalize MFR URL retrieval for new SKUs
</commit_message>
<xml_diff>
--- a/data/output/delivery_export.xlsx
+++ b/data/output/delivery_export.xlsx
@@ -1679,7 +1679,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>https://www.bosch-home.com/us/en/product/SHPM65Z55N</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
@@ -2131,7 +2135,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/us/search/searchMain/?searchkeyword=DW80R9950US</t>
+          <t>https://www.samsung.com/us/home-appliances/dishwashers/all-dishwashers/DW80R9950US/</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -2583,7 +2587,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>https://www.geappliances.com/appliance/GE-Dishwasher-GDT695SSJSS</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
@@ -3029,7 +3037,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>https://www.mieleusa.com/e/G7316SCU</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
@@ -3479,7 +3491,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>https://www.lg.com/us/dishwashers/lg-ldfn4542d/</t>
+        </is>
+      </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix dashboard event loop freezing, CORS configuration, and enforce strict HTTP 200 MFR URL verification
</commit_message>
<xml_diff>
--- a/data/output/delivery_export.xlsx
+++ b/data/output/delivery_export.xlsx
@@ -1717,22 +1717,22 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>SHPM65Z55N Bosch 500 Series 24 Inch Built-In Dishwasher 44 dBA 120V 12A Stainless Steel</t>
+          <t>SHPM65Z55N Bosch 500 Series Dishwasher SS</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>-- Unbranded --</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>-- No Unilog Brand --</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>-- No DIB Brand --</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>DISHWASHER BLTLN SST SST 120V 12A 44DBA</t>
+          <t>DISHWASHER BLTLN SST SST 120V 15A</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Bosch® Dishwasher, 500 Series, 120 V, 12 A, Built-in Mounting, 44 dBA Sound Level, Stainless Steel, Stainless Steel</t>
+          <t>Bosch® Dishwasher, 500 Series, 120 V, 15 A, Built-in Mounting, Stainless Steel, Stainless Steel</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="BQ2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="BR2" t="inlineStr">
@@ -1928,16 +1928,8 @@
           <t>Sound Level</t>
         </is>
       </c>
-      <c r="CL2" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="CM2" t="inlineStr">
-        <is>
-          <t>dBA</t>
-        </is>
-      </c>
+      <c r="CL2" t="inlineStr"/>
+      <c r="CM2" t="inlineStr"/>
       <c r="CN2" t="inlineStr">
         <is>
           <t>Material</t>
@@ -2135,7 +2127,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/us/home-appliances/dishwashers/all-dishwashers/DW80R9950US/</t>
+          <t>https://www.samsung.com/us/support/model/DW80R9950US/AA/</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -2171,22 +2163,22 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>DW80R9950US Samsung Linear Wash 24 in Top Control Built In Dishwasher 39 dBA 120V 15A Stainless Steel</t>
+          <t>DW80R9950US Samsung Dishwasher SS - Display Only</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>-- Unbranded --</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>-- No Unilog Brand --</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>-- No DIB Brand --</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -2218,27 +2210,27 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Samsung, Dishwasher, Linear Wash, DW80R9950US, Built-in Mounting</t>
+          <t>Samsung, Dishwasher, Dishwasher, DW80R9950US, Built-in Mounting</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>DISHWASHER BLTLN SST SST 120V 15A 39DBA</t>
+          <t>DISHWASHER BLTLN SST SST 120V 15A</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Samsung® Linear Wash DW80R9950US Dishwasher, Built-in Mounting, Stainless Steel</t>
+          <t>Samsung® DW80R9950US Dishwasher, Built-in Mounting, Stainless Steel</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Samsung® Dishwasher, Linear Wash, 120 V, 15 A, Built-in Mounting, 39 dBA Sound Level, Stainless Steel, Stainless Steel</t>
+          <t>Samsung® Dishwasher, 120 V, 15 A, Built-in Mounting, Stainless Steel, Stainless Steel</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Linear Wash Dishwasher, Built-in Mounting, Stainless Steel, Stainless Steel</t>
+          <t>Dishwasher, Built-in Mounting, Stainless Steel, Stainless Steel</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr"/>
@@ -2281,11 +2273,7 @@
           <t>Series</t>
         </is>
       </c>
-      <c r="BE3" t="inlineStr">
-        <is>
-          <t>Linear Wash</t>
-        </is>
-      </c>
+      <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="inlineStr">
         <is>
@@ -2382,16 +2370,8 @@
           <t>Sound Level</t>
         </is>
       </c>
-      <c r="CL3" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="CM3" t="inlineStr">
-        <is>
-          <t>dBA</t>
-        </is>
-      </c>
+      <c r="CL3" t="inlineStr"/>
+      <c r="CM3" t="inlineStr"/>
       <c r="CN3" t="inlineStr">
         <is>
           <t>Material</t>
@@ -2587,11 +2567,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>https://www.geappliances.com/appliance/GE-Dishwasher-GDT695SSJSS</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
@@ -2625,37 +2601,37 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>GDT695SSJSS GE 24 Inch Built In Dishwasher 48 dBA 120V 15A Stainless Steel</t>
+          <t>GDT695SSJSS GE Dishwasher SS</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
+          <t>-- Unbranded --</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-- No Unilog Brand --</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-- No DIB Brand --</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Appliance Dealers Cooperative (APPDE)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
           <t>GE Appliances</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>GE Appliances</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>GE</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Fastenal Company</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>GE Appliances</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>GE Appliances</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -2672,22 +2648,22 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>GE Appliances, Dishwasher, Dishwasher, GDT695SSJSS, Built-in Mounting</t>
+          <t>GE, Dishwasher, Dishwasher, GDT695SSJSS, Built-in Mounting</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>DISHWASHER BLTLN SST SST 120V 15A 48DBA</t>
+          <t>DISHWASHER BLTLN SST SST 120V 15A</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>GE Appliances® GDT695SSJSS Dishwasher, Built-in Mounting, Stainless Steel</t>
+          <t>GE® GDT695SSJSS Dishwasher, Built-in Mounting, Stainless Steel</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>GE Appliances® Dishwasher, 120 V, 15 A, Built-in Mounting, 48 dBA Sound Level, Stainless Steel, Stainless Steel</t>
+          <t>GE® Dishwasher, 120 V, 15 A, Built-in Mounting, Stainless Steel, Stainless Steel</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -2832,16 +2808,8 @@
           <t>Sound Level</t>
         </is>
       </c>
-      <c r="CL4" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="CM4" t="inlineStr">
-        <is>
-          <t>dBA</t>
-        </is>
-      </c>
+      <c r="CL4" t="inlineStr"/>
+      <c r="CM4" t="inlineStr"/>
       <c r="CN4" t="inlineStr">
         <is>
           <t>Material</t>
@@ -3037,11 +3005,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>https://www.mieleusa.com/e/G7316SCU</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
@@ -3075,27 +3039,27 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>G7316SCU Miele 24 Inch Built In Dishwasher AutoDos 42 dBA 120V 15A Clean Touch Steel</t>
+          <t>G7316SCU Miele Dishwasher SS</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Miele</t>
+          <t>-- Unbranded --</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Miele</t>
+          <t>-- No Unilog Brand --</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Miele</t>
+          <t>-- No DIB Brand --</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Grainger Industrial Supply</t>
+          <t>Freud Inc (2435)</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -3122,27 +3086,27 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>Miele, Dishwasher, Autodos, G7316SCU, Built-in Mounting</t>
+          <t>Miele, Dishwasher, Dishwasher, G7316SCU, Built-in Mounting</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>DISHWASHER BLTLN SST 120V 15A 42DBA</t>
+          <t>DISHWASHER BLTLN SST SST 120V 15A</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>Miele® Autodos G7316SCU Dishwasher, Built-in Mounting, Stainless Steel, Clean Touch Steel</t>
+          <t>Miele® G7316SCU Dishwasher, Built-in Mounting, Stainless Steel</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>Miele® Dishwasher, Autodos, 120 V, 15 A, Built-in Mounting, 42 dBA Sound Level, Stainless Steel, Clean Touch Steel</t>
+          <t>Miele® Dishwasher, 120 V, 15 A, Built-in Mounting, Stainless Steel, Stainless Steel</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>Autodos Dishwasher, Built-in Mounting, Stainless Steel, Clean Touch Steel</t>
+          <t>Dishwasher, Built-in Mounting, Stainless Steel, Stainless Steel</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr"/>
@@ -3185,11 +3149,7 @@
           <t>Series</t>
         </is>
       </c>
-      <c r="BE5" t="inlineStr">
-        <is>
-          <t>Autodos</t>
-        </is>
-      </c>
+      <c r="BE5" t="inlineStr"/>
       <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="inlineStr">
         <is>
@@ -3286,16 +3246,8 @@
           <t>Sound Level</t>
         </is>
       </c>
-      <c r="CL5" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="CM5" t="inlineStr">
-        <is>
-          <t>dBA</t>
-        </is>
-      </c>
+      <c r="CL5" t="inlineStr"/>
+      <c r="CM5" t="inlineStr"/>
       <c r="CN5" t="inlineStr">
         <is>
           <t>Material</t>
@@ -3314,7 +3266,7 @@
       </c>
       <c r="CR5" t="inlineStr">
         <is>
-          <t>Clean Touch Steel</t>
+          <t>Stainless Steel</t>
         </is>
       </c>
       <c r="CS5" t="inlineStr"/>
@@ -3493,7 +3445,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.lg.com/us/dishwashers/lg-ldfn4542d/</t>
+          <t>https://www.lg.com/us/support/product/lg-LDFN4542D</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -3529,27 +3481,27 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>LDFN4542D LG Front Control Dishwasher QuadWash 50 dBA 120V 15A Black Stainless Steel</t>
+          <t>LDFN4542D LG Dishwasher BSS</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>-- Unbranded --</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>-- No Unilog Brand --</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>-- No DIB Brand --</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>MSC Industrial Supply</t>
+          <t>Jam Industrial Supply LLC (JAMIN)</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -3576,27 +3528,27 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>LG, Dishwasher, Quadwash, LDFN4542D, Built-in Mounting</t>
+          <t>LG, Dishwasher, QuadWash Series, LDFN4542D, Built-in Mounting</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>DISHWASHER BLTLN SST SST 120V 15A 50DBA</t>
+          <t>DISHWASHER BLTLN SST SST 120V 15A</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>LG® Quadwash LDFN4542D Dishwasher, Built-in Mounting, Black Stainless Steel</t>
+          <t>LG® QuadWash Series LDFN4542D Dishwasher, Built-in Mounting, Black Stainless Steel</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>LG® Dishwasher, Quadwash, 120 V, 15 A, Built-in Mounting, 50 dBA Sound Level, Black Stainless Steel, Black Stainless Steel</t>
+          <t>LG® Dishwasher, QuadWash Series, 120 V, 15 A, Built-in Mounting, Black Stainless Steel, Black Stainless Steel</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Quadwash Dishwasher, Built-in Mounting, Black Stainless Steel, Black Stainless Steel</t>
+          <t>QuadWash Series Dishwasher, Built-in Mounting, Black Stainless Steel, Black Stainless Steel</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr"/>
@@ -3641,7 +3593,7 @@
       </c>
       <c r="BE6" t="inlineStr">
         <is>
-          <t>Quadwash</t>
+          <t>QuadWash Series</t>
         </is>
       </c>
       <c r="BF6" t="inlineStr"/>
@@ -3740,16 +3692,8 @@
           <t>Sound Level</t>
         </is>
       </c>
-      <c r="CL6" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="CM6" t="inlineStr">
-        <is>
-          <t>dBA</t>
-        </is>
-      </c>
+      <c r="CL6" t="inlineStr"/>
+      <c r="CM6" t="inlineStr"/>
       <c r="CN6" t="inlineStr">
         <is>
           <t>Material</t>

</xml_diff>

<commit_message>
Fix false LG brand resolution: exclude part numbers from brand corpus and require appliance context for bare LG token
</commit_message>
<xml_diff>
--- a/data/output/delivery_export.xlsx
+++ b/data/output/delivery_export.xlsx
@@ -9552,12 +9552,12 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>LG Electronics</t>
+          <t>UNRESOLVED — needs manual review</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>UNRESOLVED — needs manual review</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -9574,7 +9574,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>LG, Uncategorized, SF-3001</t>
+          <t>UNRESOLVED — needs manual review, Uncategorized, SF-3001</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
@@ -9584,12 +9584,12 @@
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>LG SF-3001 Uncategorized</t>
+          <t>UNRESOLVED — needs manual review SF-3001 Uncategorized</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>LG Uncategorized, SF-3001</t>
+          <t>UNRESOLVED — needs manual review Uncategorized, SF-3001</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -12240,12 +12240,12 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>LG Electronics</t>
+          <t>UNRESOLVED — needs manual review</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>UNRESOLVED — needs manual review</t>
         </is>
       </c>
       <c r="T33" t="inlineStr"/>
@@ -12262,7 +12262,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>LG, Power Tools, LG-7001</t>
+          <t>UNRESOLVED — needs manual review, Power Tools, LG-7001</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
@@ -12272,12 +12272,12 @@
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>LG LG-7001 Power Tools, 40</t>
+          <t>UNRESOLVED — needs manual review LG-7001 Power Tools, 40</t>
         </is>
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>LG Power Tools, LG-7001, 40</t>
+          <t>UNRESOLVED — needs manual review Power Tools, LG-7001, 40</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
@@ -12578,12 +12578,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>LG Electronics</t>
+          <t>UNRESOLVED — needs manual review</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>UNRESOLVED — needs manual review</t>
         </is>
       </c>
       <c r="T34" t="inlineStr"/>
@@ -12600,7 +12600,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>LG, Power Tools, LG-7002</t>
+          <t>UNRESOLVED — needs manual review, Power Tools, LG-7002</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -12610,12 +12610,12 @@
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>LG LG-7002 Power Tools, 40</t>
+          <t>UNRESOLVED — needs manual review LG-7002 Power Tools, 40</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>LG Power Tools, LG-7002, 40</t>
+          <t>UNRESOLVED — needs manual review Power Tools, LG-7002, 40</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">

</xml_diff>